<commit_message>
defined and tested all extract methods
</commit_message>
<xml_diff>
--- a/template_codebook.xlsx
+++ b/template_codebook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joemo\Desktop\oasis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91F498B7-2C67-4DE3-A1BB-53A61B0F4BF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3CE23CE-272A-4AC4-A60B-2FC939C17520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="610" yWindow="-110" windowWidth="18700" windowHeight="12220" xr2:uid="{83F1D723-4CC8-43E2-B822-F43D83F96EDB}"/>
   </bookViews>
@@ -85,9 +85,6 @@
     <t>AA01</t>
   </si>
   <si>
-    <t>12, 19, 30, 60, Inf</t>
-  </si>
-  <si>
     <t>Heat - Check Frequency</t>
   </si>
   <si>
@@ -179,6 +176,9 @@
   </si>
   <si>
     <t>reference</t>
+  </si>
+  <si>
+    <t>0, 12, 19, 30, 60, Inf</t>
   </si>
 </sst>
 </file>
@@ -605,12 +605,12 @@
         <v>8</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
         <v>10</v>
@@ -627,10 +627,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
         <v>20</v>
-      </c>
-      <c r="B4" t="s">
-        <v>21</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
@@ -647,13 +647,13 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
         <v>7</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E5" t="s">
         <v>12</v>
@@ -664,10 +664,10 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
         <v>17</v>
-      </c>
-      <c r="C6" t="s">
-        <v>18</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
@@ -724,7 +724,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>12</v>
@@ -747,73 +747,73 @@
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="2"/>
       <c r="B5" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="2"/>
       <c r="B6" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="2"/>
       <c r="B8" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="2"/>
       <c r="B9" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="2"/>
       <c r="B11" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="2"/>
       <c r="B13" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
       <c r="B14" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
       <c r="B15" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="2"/>
       <c r="B16" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -835,103 +835,103 @@
         <v>3</v>
       </c>
       <c r="B1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>